<commit_message>
feat: add Kishan Kumar (1DBSCCS103) to data/CSE.xlsx
</commit_message>
<xml_diff>
--- a/data/CSE.xlsx
+++ b/data/CSE.xlsx
@@ -52012,7 +52012,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T1001"/>
+  <dimension ref="A2:T1002"/>
   <sheetData>
     <row r="2">
       <c r="C2" t="str">
@@ -56039,41 +56039,35 @@
         <v>nie.rafi@gmail.com</v>
       </c>
     </row>
+    <row r="1002">
+      <c r="A1002">
+        <v>1001</v>
+      </c>
+      <c r="B1002" t="str">
+        <v>KISHAN KUMAR</v>
+      </c>
+      <c r="C1002" t="str">
+        <v>1DBSCCS103</v>
+      </c>
+      <c r="D1002" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="E1002" t="str">
+        <v/>
+      </c>
+      <c r="F1002" t="str">
+        <v>9739866735</v>
+      </c>
+      <c r="G1002" t="str">
+        <v/>
+      </c>
+      <c r="H1002" t="str">
+        <v>kishankumarkishan2005@gmail.com</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="C2:K3"/>
-    <mergeCell ref="C4:K4"/>
-    <mergeCell ref="C5:K5"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:O7"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="H11" r:id="rId1"/>
-    <hyperlink ref="H36" r:id="rId2"/>
-    <hyperlink ref="I44" r:id="rId3"/>
-    <hyperlink ref="I58" r:id="rId4"/>
-    <hyperlink ref="I80" r:id="rId5"/>
-    <hyperlink ref="I83" r:id="rId6"/>
-    <hyperlink ref="I86" r:id="rId7"/>
-    <hyperlink ref="I91" r:id="rId8"/>
-    <hyperlink ref="I97" r:id="rId9"/>
-    <hyperlink ref="I101" r:id="rId10"/>
-    <hyperlink ref="I103" r:id="rId11"/>
-    <hyperlink ref="I106" r:id="rId12"/>
-    <hyperlink ref="H116" r:id="rId13"/>
-    <hyperlink ref="I117" r:id="rId14"/>
-    <hyperlink ref="I119" r:id="rId15"/>
-    <hyperlink ref="H128" r:id="rId16"/>
-    <hyperlink ref="H129" r:id="rId17"/>
-    <hyperlink ref="I144" r:id="rId18"/>
-    <hyperlink ref="I149" r:id="rId19"/>
-    <hyperlink ref="H151" r:id="rId20"/>
-    <hyperlink ref="H152" r:id="rId21"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T1001"/>
+    <ignoredError numberStoredAsText="1" sqref="A2:T1002"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>